<commit_message>
feat(mexc): nativen Belegimport mit Konto- und Dublettenschutz implementieren
</commit_message>
<xml_diff>
--- a/frontend/public/import-vorlagen/import-vorlagen.xlsx
+++ b/frontend/public/import-vorlagen/import-vorlagen.xlsx
@@ -12,8 +12,9 @@
     <sheet name="bitget" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="pionex" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="coinbase" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="helium" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="solana_rpc" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mexc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="helium" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="solana_rpc" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,6 +766,60 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Creation Time(UTC+01:00)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Transaction Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -809,7 +864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
release: prepare Steuerreport V2 0.2.0rc36
</commit_message>
<xml_diff>
--- a/frontend/public/import-vorlagen/import-vorlagen.xlsx
+++ b/frontend/public/import-vorlagen/import-vorlagen.xlsx
@@ -12,8 +12,9 @@
     <sheet name="bitget" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="pionex" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="coinbase" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="helium" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="solana_rpc" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mexc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="helium" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="solana_rpc" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,6 +766,60 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Creation Time(UTC+01:00)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Transaction Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -809,7 +864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
release: prepare Steuerreport V2 0.2.0rc36 (#25)
* release: prepare Steuerreport V2 0.2.0rc36

* fix(import): expose MEXC configuration before preview

* docs(release): clarify rc36 import behavior

* test(history): align browser fixture with earn request contract

* test(history): accept explicit Earn option in browser bridge

* test(history): allow explicit Earn flag in provider probe

* test: fix rc36 CI fixtures

---------

Co-authored-by: root <root@ai-control.home.local>
</commit_message>
<xml_diff>
--- a/frontend/public/import-vorlagen/import-vorlagen.xlsx
+++ b/frontend/public/import-vorlagen/import-vorlagen.xlsx
@@ -12,8 +12,9 @@
     <sheet name="bitget" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="pionex" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="coinbase" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="helium" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="solana_rpc" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mexc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="helium" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="solana_rpc" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,6 +766,60 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Creation Time(UTC+01:00)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Transaction Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -809,7 +864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>